<commit_message>
Calendar: add Will's Prerequisites column (Knight / Math Methods pointers)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -457,23 +457,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,45 +506,55 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Prerequisites</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>HW Due</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Exams</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Topics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Reading Due</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Prerequisites</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>HW Due</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Exams</t>
         </is>
@@ -570,35 +582,41 @@
           <t>Ch. 1</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 3 (Vectors), Ch. 4-6 (Forces)</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="n">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="K2" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Fri Oct 30</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Constrained systems; generalized coordinates</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>7.2-7.3</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>HW08</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -624,33 +642,41 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Knight: Ch. 3 (Vectors), Ch. 4-6 (Forces)
+Math Methods: Ch. 5 (Cylindrical and Spherical Coordinates)
+Other: Algebra</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>HW01</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="n">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="K3" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 2</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Examples of Lagrange's equations; Lagrange multipliers</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>7.5, 7.9</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -674,31 +700,43 @@
           <t>2.1-2.2</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 5 (Drag)
+Math Methods: Ch. 1 (Intro to ODEs)
+Other: Algebra, graphs, integrals, derivatives</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="n">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="K4" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 4</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Central forces; reduced mass; equations of motion</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>8.1-8.4</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 12 (Gravity)</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -722,35 +760,48 @@
           <t>2.3-2.4</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 4 (Kinematics in 2D)
+Math Methods: Ch. 1 (Intro to ODEs)
+Other: Algebra, graphs, integrals, derivatives</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="n">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="K5" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 6</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Orbits</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>8.5-8.6</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 1 (ODEs)
+Calculus I &amp; II</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>HW09</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -776,29 +827,37 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>Knight: Ch. 3 (Vectors), Ch. 22-23 (Electromagnetism Review)
+Math Methods: Ch. 3 (Complex numbers, Euler's equation), Ch. 8 (Vector Calculus)
+Other: Cross products</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>HW02</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="I6" s="3" t="n">
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="J6" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="K6" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Mon Nov 9</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>EXAM 2 (Ch 5-7)</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr"/>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>EXAM 2 (Ch 5-7)</t>
         </is>
@@ -826,31 +885,42 @@
           <t>3.1-3.2</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 11 (Impulse and Momentum)
+Other: Integrals, vector components</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="n">
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 11</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Changing orbits</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>8.7-8.8</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Calculus I &amp; II</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -874,31 +944,38 @@
           <t>3.3-3.4</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 11 (Momentum), Ch. 12 (Rotation)
+Other: Integrals, vector components, cross products</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="n">
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="K8" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 13</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Catch-up day</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>HW10</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -924,33 +1001,44 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Knight: Ch. 12 (Rotation of Rigid Body)
+Other: Integrals, vector components</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>HW03</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="n">
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 16</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Accelerating frames; tides</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>9.1-9.2</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 8 (Vector Calculus)</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -974,31 +1062,42 @@
           <t>4.1-4.3</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 9-10 (Work and Kinetic Energy)
+Math Methods: Ch. 8 (Line integrals, curls)</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="n">
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="K10" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 18</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Angular velocity; rotating frames</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>9.3-9.5</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 8 (Vectors in Curvilinear Coordinates)</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1022,35 +1121,42 @@
           <t>4.4-4.7</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 9-10 (Potential Energy)
+Other: Full derivatives and chain rule</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="n">
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="K11" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Centrifugal force; Coriolis force</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>9.6-9.7</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>HW11</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1076,33 +1182,46 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>Knight: Ch. 12 (Gravity)
+Math Methods: Ch. 5 (Spherical Coordinates), Ch. 8 (Gradients in spherical)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>HW04</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="n">
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="K12" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 23</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Coupled oscillators; two masses and three springs</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>11.1-11.2</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 15 (Oscillations)
+Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)
+Review the ideas behind basis vectors</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1124,21 +1243,23 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="I13" s="4" t="n"/>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Wed Nov 25</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1162,23 +1283,30 @@
           <t>5.1-5.2</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Knight: Ch. 15 (Oscillations)
+Math Methods: Ch. 6 (Oscillations)</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="I14" s="4" t="n"/>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Fri Nov 27</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1204,33 +1332,43 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>Math Methods: Ch. 1 (ODEs)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
           <t>HW05</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="n">
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K15" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 30</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Normal coordinates; weakly coupled oscillators</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>11.2-11.4</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 6 (Eigenvectors/Eigenvalues)</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1248,25 +1386,27 @@
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr"/>
-      <c r="I16" s="2" t="n">
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Wed Dec 2</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Catch-up day</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1290,35 +1430,41 @@
           <t>5.5-5.6</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 3 (Complex Numbers), Ch. 1 (ODEs)</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="n">
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Fri Dec 4</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Double pendulum</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>11.4</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>HW12</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1344,29 +1490,35 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>Math Methods: Ch. 9 (Fourier Series and Transforms)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>HW06</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="I18" s="3" t="n">
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="J18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="J18" s="3" t="n">
+      <c r="K18" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>Mon Dec 7</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>EXAM 3 (Ch 8, 9, 11)</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr"/>
       <c r="N18" s="3" t="inlineStr"/>
-      <c r="O18" s="3" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr"/>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>EXAM 3 (Ch 8, 9, 11)</t>
         </is>
@@ -1391,34 +1543,36 @@
       </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>EXAM 1 (Ch 2-4)</t>
         </is>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="J19" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="K19" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Wed Dec 9</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Chaos</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>12.1-12.3</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1442,35 +1596,41 @@
           <t>6.1-6.2</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 4 (Partial Derivatives), Ch. 5 (Integration)</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="n">
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="K20" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Fri Dec 11</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Chaos</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>12.1-12.3</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>HW13</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1496,29 +1656,35 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
+          <t>Math Methods: Ch. 4 (Partial Derivatives)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
           <t>HW07</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="n">
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="K21" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 14</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Last day: review and wrap-up</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1544,21 +1710,23 @@
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="I22" s="4" t="n"/>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (registrar schedules)</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
       <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>Final (Ch 12 required + optional grade-replacement)</t>
         </is>
@@ -1588,6 +1756,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
F2026: PCCIs for every class day; 1.50 starter notebook; TODO state
PCCI column filled from Will's Look-At problems (one per day, easiest
star where he listed two; reading prompts where he had none). New
NewtonsLaws/skateboard_1_50.ipynb: Python port of the HW01 computational
problem (full vs small-angle pendulum, period vs amplitude), executed.
TODO records prep packs 01-05 done and the Ch 3-4 errata headlines.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -587,7 +587,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Read the syllabus; bring one question or comment</t>
+          <t>Read the syllabus and bring one question or comment; and 1.10</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -622,7 +622,11 @@
 Other: Algebra, graphs, integrals, derivatives</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
@@ -655,7 +659,11 @@
 Other: Algebra, graphs, integrals, derivatives</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>HW01</t>
@@ -692,7 +700,11 @@
 Other: Cross products</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2.49</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
     </row>
@@ -724,7 +736,11 @@
 Other: Integrals, vector components</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +772,11 @@
 Other: Integrals, vector components, cross products</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>HW02</t>
@@ -792,7 +812,11 @@
 Other: Integrals, vector components</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>3.32</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
@@ -824,7 +848,11 @@
 Math Methods: Ch. 8 (Line integrals, curls)</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -856,7 +884,11 @@
 Other: Full derivatives and chain rule</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>4.31</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>HW03</t>
@@ -892,7 +924,11 @@
 Math Methods: Ch. 5 (Spherical Coordinates), Ch. 8 (Gradients in spherical)</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>4.41</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -915,7 +951,11 @@
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Bring one Ch 1-4 problem you want worked in the problem session (skip if Mountain Day)</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
F2026: Noether's theorem via Taylor 7.8 on Nov 2; 7.46 on HW09
Michael asked for a simple version of Noether's theorem. Taylor 7.8 is
exactly that (translation invariance -> momentum; time independence ->
Hamiltonian), so it joins the Mon Nov 2 reading, and 7.46 (rotational
invariance -> L_z) joins HW09. Reading label 7.9 -> 7.10 for Lagrange
multipliers (Taylor's 7.9 is magnetic forces); flagged in TODO.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -1386,12 +1386,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Examples of Lagrange's equations; Lagrange multipliers</t>
+          <t>Examples of Lagrange's equations; Noether's theorem (symmetries and conservation laws); Lagrange multipliers</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>7.5, 7.9</t>
+          <t>7.5, 7.8, 7.10</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>7.5, 7.9, 8.1-8.2: Lagrangian examples; multipliers; two-body setup</t>
+          <t>7.5, 7.8, 7.9, 8.1-8.2: Lagrangian examples; Noether; multipliers; two-body setup</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>7.27, 7.31, 7.34, 7.38 [optional challenge], 8.2</t>
+          <t>7.27, 7.31, 7.34, 7.38 [optional challenge], 7.46 [Noether: rotational invariance gives conservation of L_z], 8.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coverage audit against Taylor's section headers; three readings widened
audit_taylor_coverage.py: every assigned problem -> its Taylor section
(from OCR of the scanned book's problem pages) -> the first class day
whose reading covers it -> compared with the due date. 71 problems,
0 violations after widening Ch 2 day 3 to 2.5-2.7, Ch 9 day 3 to
9.6-9.8, and the chaos days to 12.1-12.4 / 12.4-12.5, which is what
Will taught on those days; his labels were narrower.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.5-2.7</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>9.6-9.7</t>
+          <t>9.6-9.8</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>12.1-12.3</t>
+          <t>12.1-12.4</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>12.1-12.3</t>
+          <t>12.4-12.5</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
F2026: exams Fri Oct 9 / Wed Nov 11; 60-pt exam problems; chapter problem lists
Michael's revisions (2026-09-04): each exam after the last homework on
its chapters is returned, so Exam 1 moves to Fri Oct 9 (Will's slot;
HW04 due Mon Oct 5) and Exam 2 to Wed Nov 11 (HW09 due Fri Nov 6, back
on the Mon Nov 9 review day). Grading: PCCIs 3.2 x 35 = 112, HW 24 x 12
= 288, exams 3 x 180, final 60 -- every exam-type problem exactly 60.
Generator: EXAMS indices, HW dates, PCCI moves, cats; new CHAPTER_PROBLEMS
data -> "Chapter Problems" tab + ChapterProblemLists.md (Look at / In
class / Homework per chapter, the chapter-opening slide). Syllabus key
dates updated (Michael's grading table and exam-paragraph edits kept;
one typo fixed). Coverage audit: 0 violations. TODO lists the Moodle
hand edits the live course now needs.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY317 F2026 Calendar.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Problems" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45,12 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -956,7 +957,11 @@
           <t>Bring one Ch 1-4 problem you want worked in the problem session (skip if Mountain Day)</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>HW04</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
@@ -992,66 +997,54 @@
           <t>5.1</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>HW04</t>
-        </is>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Fri Oct 9</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2D oscillators; damped SHO</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>5.3-5.4</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Math Methods: Ch. 1 (ODEs)</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>5.21</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>EXAM 1 (Ch 2-4)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>EXAM 1 (Ch 2-4)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Mon Oct 12</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>No class - Autumn recess</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1114,22 +1107,22 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Forced damped SHO; resonance</t>
+          <t>2D oscillators; damped SHO</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>5.5-5.6</t>
+          <t>5.3-5.4</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Math Methods: Ch. 3 (Complex Numbers), Ch. 1 (ODEs)</t>
+          <t>Math Methods: Ch. 1 (ODEs)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>5.35</t>
+          <t>5.21</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1153,53 +1146,61 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Fourier series analysis of driven SHO</t>
+          <t>Forced damped SHO; resonance</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>5.7-5.8</t>
+          <t>5.5-5.6</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Math Methods: Ch. 9 (Fourier Series and Transforms)</t>
+          <t>Math Methods: Ch. 3 (Complex Numbers), Ch. 1 (ODEs)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>5.47</t>
+          <t>5.35</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Mon Oct 19</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>EXAM 1 (Ch 2-4)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>EXAM 1 (Ch 2-4)</t>
-        </is>
-      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Fourier series analysis of driven SHO</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>5.7-5.8</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Math Methods: Ch. 9 (Fourier Series and Transforms)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>5.47</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1475,7 +1476,11 @@
           <t>8.19</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>HW09</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1492,84 +1497,80 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Changing orbits</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>8.7-8.8</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Calculus I &amp; II</t>
-        </is>
-      </c>
+          <t>Catch-up / review day (Exam 2 is Wednesday)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>8.28</t>
+          <t>Bring one Ch 5-7 problem you want worked in review</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Wed Nov 11</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Catch-up / review day (Exam 2 is Friday)</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Bring one Ch 5-7 problem you want worked in review</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>HW09</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>EXAM 2 (Ch 5-7)</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>EXAM 2 (Ch 5-7)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 13</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>EXAM 2 (Ch 5-7)</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>EXAM 2 (Ch 5-7)</t>
-        </is>
-      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Changing orbits</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>8.7-8.8</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Calculus I &amp; II</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>8.28</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1718,42 +1719,42 @@
       <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n"/>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Wed Nov 25</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Fri Nov 27</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1853,27 +1854,27 @@
       <c r="I40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B41" s="4" t="n">
+      <c r="B41" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Mon Dec 7</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>EXAM 3 (Ch 8, 9, 11)</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>EXAM 3 (Ch 8, 9, 11)</t>
         </is>
@@ -1969,46 +1970,46 @@
       <c r="I44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n"/>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Wed Dec 16</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Reading period</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>HW13</t>
         </is>
       </c>
-      <c r="I45" s="3" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="A46" s="4" t="n"/>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (self-scheduled)</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>Final (Ch 12 required + optional grade-replacement)</t>
         </is>
@@ -2158,7 +2159,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 7</t>
+          <t>Mon Oct 5</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2190,7 +2191,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.4: SHO, 2D oscillators, damping</t>
+          <t>5.1-5.2: Hooke's law, simple harmonic motion</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2217,7 +2218,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>5.5-5.8: driven oscillators, resonance, Fourier series</t>
+          <t>5.3-5.8: 2D and damped oscillators, resonance, Fourier series</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2293,7 +2294,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 11</t>
+          <t>Fri Nov 6</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2484,7 +2485,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="E2">
         <f>(B2-C2)*D2</f>
@@ -2504,7 +2505,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E3">
         <f>(B3-C3)*D3</f>
@@ -2524,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="E4">
         <f>(B4-C4)*D4</f>
@@ -2561,6 +2562,690 @@
         <f>SUM(E2:E5)</f>
         <v/>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Chapter</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Look at (PCCI source)</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>In class</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>1.4, 1.6, 1.10, 1.11, 1.31, 1.35</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1.9, 1.18, 1.26, 1.43, 1.47, 1.48</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>HW01: 1.27, 1.45, 1.46, 1.49, 1.50 (computational)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>2.1, 2.5, 2.7</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>2.4, 2.11, 2.12, 2.13</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>HW02: 2.14, 2.31, 2.36, 2.39, 2.42, 2.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>2.16, 2.25</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2.33, 2.34, 2.35, 2.41</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>2.49</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2.52, 2.54</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>3.5, 3.10, 3.11</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>HW03: 3.8, 3.13, 3.19, 3.35, 3.36, Challenge: chain lifted at constant speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>3.16, 3.17, 3.25</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>3.21, 3.27</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>3.32</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>3.29, 3.34</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>4.7, 4.16</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>4.2, 4.3, 4.12, 4.15</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>HW04: 4.4, 4.8, 4.13 (optional), 4.24(a-c), Variation of gravity with height, 4.36, 4.39 (advanced, optional), 4.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>4.31</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>4.23, 4.26, 4.28</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>4.41</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>4.46, 4.48</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>5.1, 5.3</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>5.6, 5.8, 5.12</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>HW05: 5.4, 5.7, 5.13
+HW06: 5.28, 5.32 (optional), 5.43, RLC circuit as an SHO, Square-wave drive (or 5.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>5.21</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>5.22, 5.26</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>5.35</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>5.40, 5.41, 5.42, 5.44</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Day 4</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>5.47</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>5.49</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>6.3, 6.4</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>6.1, 6.2</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>HW07: 6.7, 6.11, 6.14, 6.17, Brachistochrone revisited
+HW08: 6.23, 6.24 (advanced, optional), 6.27</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>6.9, 6.18</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>6.20</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>6.21, 6.25</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>7.1, 7.2</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>7.4, 7.8</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>HW08: 7.3, 7.10, 7.14
+HW09: 7.27, 7.31, 7.34, 7.38 (optional challenge), 7.46 (Noether)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>7.17, 7.19</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>7.20, 7.33, 7.36</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>8.6, 8.8</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>8.3, 8.10</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>HW09: 8.2
+HW10: 8.9, 8.13, 8.14 (optional challenge), 8.15, 8.18, 8.23
+HW11: 8.27 (optional challenge), 8.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>8.19, 8.20</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>8.12, 8.21</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>8.28, 8.32</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>8.29, 8.33, 8.34</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>HW11: 9.3, 9.9, 9.15, 9.17, 9.28, 9.29 (optional challenge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>9.12, 9.13</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>9.14, 9.16, 9.19</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>11.2, 11.3</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>HW12: 11.6, 11.9, 11.12, 11.14, 11.17 (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>driven-pendulum notebook: period exploration, Poincare section</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>HW13: 12.1, 12.6, 12.7, 12.8-12.10 (optional), 12.13 + parts (b), (c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>bifurcation diagram, Lyapunov exponent</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>